<commit_message>
Updates for draft version MACC
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_Z_SYS_Additional_AssumptionsMACC.xlsx
+++ b/SuppXLS/Scen_Z_SYS_Additional_AssumptionsMACC.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rbsul\Documents\GitHub\times-ireland-model\SuppXLS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BSuleimenov\Documents\GitHub\times-ireland-model\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ED7E09C-CE5E-493F-A5E9-41958BA24DA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF2C8A27-D73E-4C66-862F-93D5B837B98E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="29" r:id="rId1"/>
@@ -11841,7 +11841,7 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>19050</xdr:colOff>
+          <xdr:colOff>22860</xdr:colOff>
           <xdr:row>3</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:to>
@@ -12300,17 +12300,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C79DA532-7D5D-4233-BA89-FC4C950C7D0C}">
   <sheetPr codeName="Sheet11"/>
   <dimension ref="A1:Z99"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="4" width="21.7109375" customWidth="1"/>
-    <col min="5" max="6" width="14.140625" customWidth="1"/>
-    <col min="7" max="7" width="12.140625" customWidth="1"/>
-    <col min="8" max="10" width="8.140625" customWidth="1"/>
-    <col min="11" max="11" width="9.7109375" customWidth="1"/>
-    <col min="12" max="12" width="8.140625" customWidth="1"/>
+    <col min="1" max="4" width="21.6640625" customWidth="1"/>
+    <col min="5" max="6" width="14.109375" customWidth="1"/>
+    <col min="7" max="7" width="12.109375" customWidth="1"/>
+    <col min="8" max="10" width="8.109375" customWidth="1"/>
+    <col min="11" max="11" width="9.6640625" customWidth="1"/>
+    <col min="12" max="12" width="8.109375" customWidth="1"/>
     <col min="13" max="13" width="10" customWidth="1"/>
-    <col min="14" max="14" width="11.42578125" customWidth="1"/>
-    <col min="15" max="15" width="13.42578125" customWidth="1"/>
+    <col min="14" max="14" width="11.44140625" customWidth="1"/>
+    <col min="15" max="15" width="13.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26">
@@ -15147,36 +15147,36 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F0F7499-A5CE-4374-995E-DC72D788363A}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A3:AD37"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="11.7109375" customWidth="1"/>
-    <col min="3" max="3" width="3.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="5.5703125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="4.85546875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="7.5703125" customWidth="1"/>
-    <col min="25" max="25" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.109375" customWidth="1"/>
+    <col min="2" max="2" width="11.6640625" customWidth="1"/>
+    <col min="3" max="3" width="3.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6.109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="6.109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="4.88671875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="7.5546875" customWidth="1"/>
+    <col min="25" max="25" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="6.109375" bestFit="1" customWidth="1"/>
     <col min="27" max="28" width="6" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="6.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:30">
@@ -15647,7 +15647,7 @@
         <v>IE-MN</v>
       </c>
     </row>
-    <row r="10" spans="1:30" ht="15.75" thickBot="1">
+    <row r="10" spans="1:30" ht="15" thickBot="1">
       <c r="A10" s="13" t="s">
         <v>23</v>
       </c>
@@ -15889,7 +15889,7 @@
                   </from>
                   <to>
                     <xdr:col>1</xdr:col>
-                    <xdr:colOff>19050</xdr:colOff>
+                    <xdr:colOff>22860</xdr:colOff>
                     <xdr:row>3</xdr:row>
                     <xdr:rowOff>0</xdr:rowOff>
                   </to>
@@ -15908,12 +15908,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FE79BAD-EA44-47F0-A194-320DE6C9FB50}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="B2:W62"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:23">
@@ -15999,7 +15999,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="2:23" ht="45">
+    <row r="6" spans="2:23" ht="43.2">
       <c r="B6" s="19" t="s">
         <v>145</v>
       </c>
@@ -16178,7 +16178,7 @@
       </c>
       <c r="M15" s="7"/>
     </row>
-    <row r="16" spans="2:23" ht="15.75" thickBot="1">
+    <row r="16" spans="2:23" ht="15" thickBot="1">
       <c r="B16" s="8" t="s">
         <v>12</v>
       </c>
@@ -16325,7 +16325,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="24" spans="2:12" ht="15.75" thickBot="1">
+    <row r="24" spans="2:12" ht="15" thickBot="1">
       <c r="B24" s="8" t="s">
         <v>12</v>
       </c>
@@ -16595,7 +16595,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="37" spans="2:12" ht="15.75" thickBot="1">
+    <row r="37" spans="2:12" ht="15" thickBot="1">
       <c r="B37" s="8" t="s">
         <v>12</v>
       </c>
@@ -17031,7 +17031,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93BCBE91-6737-4A5C-8B05-174F9388360E}">
   <dimension ref="C4:L9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="4" spans="3:12">
       <c r="C4" s="4" t="s">
@@ -17080,7 +17080,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="3:12" ht="30">
+    <row r="8" spans="3:12" ht="28.8">
       <c r="C8" s="19" t="s">
         <v>262</v>
       </c>
@@ -17130,10 +17130,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DE4666E-C19A-4073-8183-3ACBB585B13C}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="B2:J4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:10">
@@ -17144,7 +17144,7 @@
       <c r="I2" s="7"/>
       <c r="J2" s="7"/>
     </row>
-    <row r="3" spans="2:10" ht="15.75" thickBot="1">
+    <row r="3" spans="2:10" ht="15" thickBot="1">
       <c r="B3" s="8" t="s">
         <v>12</v>
       </c>
@@ -17201,19 +17201,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:V60"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="23.7109375" customWidth="1"/>
-    <col min="3" max="3" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.85546875" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" customWidth="1"/>
+    <col min="3" max="3" width="8.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.88671875" customWidth="1"/>
     <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="30.28515625" customWidth="1"/>
-    <col min="12" max="12" width="44.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="30.33203125" customWidth="1"/>
+    <col min="12" max="12" width="44.6640625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="12" customWidth="1"/>
   </cols>
   <sheetData>
@@ -17302,7 +17302,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:22" ht="30">
+    <row r="6" spans="1:22" ht="28.8">
       <c r="B6" s="38" t="s">
         <v>111</v>
       </c>
@@ -17640,7 +17640,7 @@
     </row>
     <row r="16" spans="1:22">
       <c r="H16" t="s">
-        <v>7</v>
+        <v>259</v>
       </c>
     </row>
     <row r="17" spans="2:13">
@@ -17801,7 +17801,7 @@
       <c r="I27" s="7"/>
       <c r="J27" s="7"/>
     </row>
-    <row r="28" spans="2:13" ht="15.75" thickBot="1">
+    <row r="28" spans="2:13" ht="15" thickBot="1">
       <c r="B28" s="8" t="s">
         <v>12</v>
       </c>
@@ -17890,7 +17890,7 @@
       <c r="H33" s="7"/>
       <c r="I33" s="7"/>
     </row>
-    <row r="34" spans="2:13" ht="15.75" thickBot="1">
+    <row r="34" spans="2:13" ht="15" thickBot="1">
       <c r="B34" s="8" t="s">
         <v>12</v>
       </c>
@@ -18022,7 +18022,7 @@
       <c r="K41" s="7"/>
       <c r="L41" s="7"/>
     </row>
-    <row r="42" spans="2:13" ht="15.75" thickBot="1">
+    <row r="42" spans="2:13" ht="15" thickBot="1">
       <c r="B42" s="8" t="s">
         <v>12</v>
       </c>
@@ -18072,7 +18072,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="54" spans="2:11" ht="15.75" thickBot="1">
+    <row r="54" spans="2:11" ht="15" thickBot="1">
       <c r="B54" s="19" t="s">
         <v>181</v>
       </c>
@@ -18276,10 +18276,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F532AC2E-E047-4124-A56C-AD8CA9B97A1E}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="B3:I12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:9">
@@ -18289,7 +18289,7 @@
       <c r="H3" s="7"/>
       <c r="I3" s="7"/>
     </row>
-    <row r="4" spans="2:9" ht="15.75" thickBot="1">
+    <row r="4" spans="2:9" ht="15" thickBot="1">
       <c r="B4" s="8" t="s">
         <v>12</v>
       </c>
@@ -18494,19 +18494,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8FB1178-AF9A-473D-9FB3-41C2F896D89C}">
   <sheetPr codeName="Sheet7"/>
   <dimension ref="B3:M91"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="22.85546875" customWidth="1"/>
-    <col min="3" max="3" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.85546875" customWidth="1"/>
-    <col min="5" max="6" width="11.7109375" customWidth="1"/>
-    <col min="9" max="9" width="13.42578125" customWidth="1"/>
-    <col min="10" max="10" width="14.7109375" customWidth="1"/>
-    <col min="11" max="11" width="28.42578125" customWidth="1"/>
-    <col min="12" max="12" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="22.5703125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.88671875" customWidth="1"/>
+    <col min="3" max="3" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.88671875" customWidth="1"/>
+    <col min="5" max="6" width="11.6640625" customWidth="1"/>
+    <col min="9" max="9" width="13.44140625" customWidth="1"/>
+    <col min="10" max="10" width="14.6640625" customWidth="1"/>
+    <col min="11" max="11" width="28.44140625" customWidth="1"/>
+    <col min="12" max="12" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="22.5546875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="13.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:13">
@@ -18516,7 +18516,7 @@
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
     </row>
-    <row r="4" spans="2:13" ht="15.75" thickBot="1">
+    <row r="4" spans="2:13" ht="15" thickBot="1">
       <c r="B4" s="8" t="s">
         <v>12</v>
       </c>
@@ -19527,7 +19527,7 @@
       <c r="C60" s="58"/>
       <c r="D60" s="58"/>
     </row>
-    <row r="61" spans="2:13" ht="15.75">
+    <row r="61" spans="2:13" ht="15.6">
       <c r="B61" s="58"/>
       <c r="C61" s="64">
         <v>2018</v>
@@ -19742,7 +19742,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="73" spans="2:8" ht="15.75">
+    <row r="73" spans="2:8" ht="15.6">
       <c r="B73" s="59" t="s">
         <v>214</v>
       </c>

</xml_diff>